<commit_message>
docs: documents 26/05/14_1 work
</commit_message>
<xml_diff>
--- a/doc/基本設計/01_画面一覧.xlsx
+++ b/doc/基本設計/01_画面一覧.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="29">
   <si>
     <t xml:space="preserve">■画面一覧</t>
   </si>
@@ -58,13 +58,13 @@
     <t xml:space="preserve">SCR-002</t>
   </si>
   <si>
-    <t xml:space="preserve">ホーム画面</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/home</t>
-  </si>
-  <si>
-    <t xml:space="preserve">打刻・サマリー表示</t>
+    <t xml:space="preserve">勤怠一覧画面</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/attendance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">勤怠履歴一覧</t>
   </si>
   <si>
     <t xml:space="preserve">一般</t>
@@ -73,43 +73,31 @@
     <t xml:space="preserve">SCR-003</t>
   </si>
   <si>
-    <t xml:space="preserve">勤怠一覧画面</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/attendance</t>
-  </si>
-  <si>
-    <t xml:space="preserve">勤怠履歴一覧</t>
+    <t xml:space="preserve">勤怠詳細画面</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/attendance/:id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">勤怠詳細表示</t>
   </si>
   <si>
     <t xml:space="preserve">SCR-004</t>
   </si>
   <si>
-    <t xml:space="preserve">勤怠詳細画面</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/attendance/:id</t>
-  </si>
-  <si>
-    <t xml:space="preserve">勤怠詳細表示</t>
+    <t xml:space="preserve">管理者画面</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/admin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">管理者トップ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">管理者</t>
   </si>
   <si>
     <t xml:space="preserve">SCR-005</t>
-  </si>
-  <si>
-    <t xml:space="preserve">管理者画面</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/admin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">管理者トップ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">管理者</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SCR-006</t>
   </si>
   <si>
     <t xml:space="preserve">ユーザー一覧</t>
@@ -518,7 +506,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B1:G11"/>
+  <dimension ref="B1:G1048576"/>
   <sheetFormatPr defaultColWidth="10.4921875" defaultRowHeight="13.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4.15"/>
@@ -629,44 +617,27 @@
         <v>23</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="G9" s="6"/>
+        <v>24</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="E10" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="F10" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="C10" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="D10" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="E10" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="F10" s="8" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="C11" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="D11" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="E11" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="F11" s="8" t="s">
-        <v>28</v>
-      </c>
-    </row>
+    </row>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>

</xml_diff>